<commit_message>
data: update release batch 29/29
</commit_message>
<xml_diff>
--- a/countries/cn/2026-2029.xlsx
+++ b/countries/cn/2026-2029.xlsx
@@ -51620,7 +51620,7 @@
       </c>
       <c r="AJ331" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK331" t="inlineStr">
@@ -51851,7 +51851,7 @@
       </c>
       <c r="AJ332" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK332" t="inlineStr">
@@ -52243,7 +52243,7 @@
       </c>
       <c r="AJ334" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK334" t="inlineStr">
@@ -52639,7 +52639,7 @@
       </c>
       <c r="AJ336" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK336" t="inlineStr">
@@ -53035,7 +53035,7 @@
       </c>
       <c r="AJ338" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK338" t="inlineStr">
@@ -53431,7 +53431,7 @@
       </c>
       <c r="AJ340" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK340" t="inlineStr">
@@ -53827,7 +53827,7 @@
       </c>
       <c r="AJ342" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK342" t="inlineStr">
@@ -60892,7 +60892,7 @@
       </c>
       <c r="AJ387" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK387" t="inlineStr">
@@ -62053,7 +62053,7 @@
       </c>
       <c r="AJ394" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK394" t="inlineStr">
@@ -62284,7 +62284,7 @@
       </c>
       <c r="AJ395" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK395" t="inlineStr">
@@ -62676,7 +62676,7 @@
       </c>
       <c r="AJ397" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK397" t="inlineStr">
@@ -63072,7 +63072,7 @@
       </c>
       <c r="AJ399" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK399" t="inlineStr">
@@ -63468,7 +63468,7 @@
       </c>
       <c r="AJ401" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK401" t="inlineStr">
@@ -63864,7 +63864,7 @@
       </c>
       <c r="AJ403" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK403" t="inlineStr">
@@ -64260,7 +64260,7 @@
       </c>
       <c r="AJ405" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK405" t="inlineStr">
@@ -71325,7 +71325,7 @@
       </c>
       <c r="AJ450" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK450" t="inlineStr">

</xml_diff>